<commit_message>
Add service update use case
</commit_message>
<xml_diff>
--- a/docs/Methods.xlsx
+++ b/docs/Methods.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\API\ConferenceRoomBooking\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DB8F6DD6-68AE-47DB-A8AA-ACF76C1BEA70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80672433-3294-4EDE-973C-36CEA4013C57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{290D68D7-7384-40BB-827B-CD27B026537C}"/>
+    <workbookView xWindow="-28920" yWindow="4185" windowWidth="29040" windowHeight="15720" xr2:uid="{290D68D7-7384-40BB-827B-CD27B026537C}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,10 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="35">
-  <si>
-    <t>Service</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="43">
   <si>
     <t>Method</t>
   </si>
@@ -78,9 +75,6 @@
     <t>GetByIdAsync()</t>
   </si>
   <si>
-    <t>SaveChangesAsync(</t>
-  </si>
-  <si>
     <t>SearchAvailableAsync()</t>
   </si>
   <si>
@@ -139,13 +133,43 @@
   </si>
   <si>
     <t>CreateBookingDto</t>
+  </si>
+  <si>
+    <t>SaveChangesAsync ()</t>
+  </si>
+  <si>
+    <t>Controller method</t>
+  </si>
+  <si>
+    <t>Endpoint</t>
+  </si>
+  <si>
+    <t>Create</t>
+  </si>
+  <si>
+    <t>Update</t>
+  </si>
+  <si>
+    <t>Delete</t>
+  </si>
+  <si>
+    <t>POST /api/services</t>
+  </si>
+  <si>
+    <t>PUT /api/services/{id}</t>
+  </si>
+  <si>
+    <t>DELETE /api/services/{id}</t>
+  </si>
+  <si>
+    <t>Application Service</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -165,13 +189,26 @@
       <name val="Consolas"/>
       <family val="3"/>
     </font>
+    <font>
+      <strike/>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.14999847407452621"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -201,7 +238,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -219,6 +256,15 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -538,315 +584,393 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="C3:G25"/>
+  <dimension ref="C3:I25"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="0" style="1" hidden="1" customWidth="1"/>
     <col min="3" max="3" width="24.28515625" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="23.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="36" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="37.140625" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="52.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="33.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="16384" width="9.140625" style="1"/>
+    <col min="7" max="7" width="34.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="19.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="28.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="3:7" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C3" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="D3" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="E3" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="F3" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="F3" s="3" t="s">
+      <c r="G3" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="G3" s="3" t="s">
+      <c r="H3" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="I3" s="3" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="4" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C4" s="4" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="4" spans="3:7" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C4" s="4" t="s">
+      <c r="D4" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="E4" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="F4" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="F4" s="5" t="s">
+      <c r="G4" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="G4" s="6" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="5" spans="3:7" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="H4" s="5"/>
+      <c r="I4" s="5"/>
+    </row>
+    <row r="5" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C5" s="4"/>
       <c r="D5" s="5"/>
       <c r="E5" s="5"/>
       <c r="F5" s="5"/>
       <c r="G5" s="6" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="6" spans="3:7" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+        <v>9</v>
+      </c>
+      <c r="H5" s="5"/>
+      <c r="I5" s="5"/>
+    </row>
+    <row r="6" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C6" s="4"/>
       <c r="D6" s="5"/>
       <c r="E6" s="5"/>
       <c r="F6" s="5"/>
       <c r="G6" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="H6" s="5"/>
+      <c r="I6" s="5"/>
+    </row>
+    <row r="7" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C7" s="4"/>
+      <c r="D7" s="5" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="7" spans="3:7" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C7" s="4"/>
-      <c r="D7" s="3" t="s">
+      <c r="E7" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F7" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="G7" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="E7" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="F7" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="G7" s="6" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="8" spans="3:7" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="H7" s="5"/>
+      <c r="I7" s="5"/>
+    </row>
+    <row r="8" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C8" s="4"/>
-      <c r="D8" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="E8" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="F8" s="5" t="s">
-        <v>24</v>
-      </c>
+      <c r="D8" s="5"/>
+      <c r="E8" s="5"/>
+      <c r="F8" s="5"/>
       <c r="G8" s="6" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="9" spans="3:7" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+        <v>8</v>
+      </c>
+      <c r="H8" s="5"/>
+      <c r="I8" s="5"/>
+    </row>
+    <row r="9" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C9" s="4"/>
       <c r="D9" s="5"/>
       <c r="E9" s="5"/>
       <c r="F9" s="5"/>
       <c r="G9" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="H9" s="5"/>
+      <c r="I9" s="5"/>
+    </row>
+    <row r="10" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C10" s="4"/>
+      <c r="D10" s="5" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="10" spans="3:7" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C10" s="4"/>
-      <c r="D10" s="5"/>
-      <c r="E10" s="5"/>
-      <c r="F10" s="5"/>
+      <c r="E10" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="F10" s="5" t="s">
+        <v>22</v>
+      </c>
       <c r="G10" s="6" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="11" spans="3:7" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+        <v>12</v>
+      </c>
+      <c r="H10" s="5"/>
+      <c r="I10" s="5"/>
+    </row>
+    <row r="11" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C11" s="4"/>
-      <c r="D11" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="E11" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="F11" s="5" t="s">
-        <v>25</v>
-      </c>
+      <c r="D11" s="5"/>
+      <c r="E11" s="5"/>
+      <c r="F11" s="5"/>
       <c r="G11" s="6" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="12" spans="3:7" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+      <c r="H11" s="5"/>
+      <c r="I11" s="5"/>
+    </row>
+    <row r="12" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C12" s="4"/>
       <c r="D12" s="5"/>
       <c r="E12" s="5"/>
       <c r="F12" s="5"/>
       <c r="G12" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="H12" s="5"/>
+      <c r="I12" s="5"/>
+    </row>
+    <row r="13" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C13" s="4"/>
+      <c r="D13" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="F13" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="G13" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="H13" s="3"/>
+      <c r="I13" s="3"/>
+    </row>
+    <row r="14" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C14" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="D14" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="E14" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="F14" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="G14" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="H14" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="I14" s="5" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="15" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C15" s="5"/>
+      <c r="D15" s="7"/>
+      <c r="E15" s="7"/>
+      <c r="F15" s="7"/>
+      <c r="G15" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="H15" s="5"/>
+      <c r="I15" s="5"/>
+    </row>
+    <row r="16" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C16" s="5"/>
+      <c r="D16" s="7"/>
+      <c r="E16" s="7"/>
+      <c r="F16" s="7"/>
+      <c r="G16" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="H16" s="5"/>
+      <c r="I16" s="5"/>
+    </row>
+    <row r="17" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C17" s="5"/>
+      <c r="D17" s="7" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="13" spans="3:7" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C13" s="4"/>
-      <c r="D13" s="5"/>
-      <c r="E13" s="5"/>
-      <c r="F13" s="5"/>
-      <c r="G13" s="3" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="14" spans="3:7" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C14" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="D14" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="E14" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="F14" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="G14" s="6" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="15" spans="3:7" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C15" s="5"/>
-      <c r="D15" s="5"/>
-      <c r="E15" s="5"/>
-      <c r="F15" s="5"/>
-      <c r="G15" s="6" t="s">
+      <c r="E17" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="F17" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="G17" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="H17" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="I17" s="5" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="18" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C18" s="5"/>
+      <c r="D18" s="7"/>
+      <c r="E18" s="7"/>
+      <c r="F18" s="7"/>
+      <c r="G18" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="H18" s="5"/>
+      <c r="I18" s="5"/>
+    </row>
+    <row r="19" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C19" s="5"/>
+      <c r="D19" s="7"/>
+      <c r="E19" s="7"/>
+      <c r="F19" s="7"/>
+      <c r="G19" s="9" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="16" spans="3:7" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C16" s="5"/>
-      <c r="D16" s="5"/>
-      <c r="E16" s="5"/>
-      <c r="F16" s="5"/>
-      <c r="G16" s="6" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="17" spans="3:7" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C17" s="5"/>
-      <c r="D17" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="E17" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="F17" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="G17" s="6" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="18" spans="3:7" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C18" s="5"/>
-      <c r="D18" s="5"/>
-      <c r="E18" s="5"/>
-      <c r="F18" s="5"/>
-      <c r="G18" s="6" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="19" spans="3:7" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C19" s="5"/>
-      <c r="D19" s="5"/>
-      <c r="E19" s="5"/>
-      <c r="F19" s="5"/>
-      <c r="G19" s="6" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="20" spans="3:7" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="H19" s="5"/>
+      <c r="I19" s="5"/>
+    </row>
+    <row r="20" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C20" s="5"/>
       <c r="D20" s="5" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="F20" s="5" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="G20" s="6" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="21" spans="3:7" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+        <v>12</v>
+      </c>
+      <c r="H20" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="I20" s="5" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="21" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C21" s="5"/>
       <c r="D21" s="5"/>
       <c r="E21" s="5"/>
       <c r="F21" s="5"/>
       <c r="G21" s="6" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="22" spans="3:7" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+      <c r="H21" s="5"/>
+      <c r="I21" s="5"/>
+    </row>
+    <row r="22" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C22" s="5"/>
       <c r="D22" s="5"/>
       <c r="E22" s="5"/>
       <c r="F22" s="5"/>
       <c r="G22" s="6" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="23" spans="3:7" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+        <v>10</v>
+      </c>
+      <c r="H22" s="5"/>
+      <c r="I22" s="5"/>
+    </row>
+    <row r="23" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C23" s="5" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="D23" s="5" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E23" s="5" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="F23" s="5" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="G23" s="6" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="24" spans="3:7" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+        <v>18</v>
+      </c>
+      <c r="H23" s="5"/>
+      <c r="I23" s="5"/>
+    </row>
+    <row r="24" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C24" s="5"/>
       <c r="D24" s="5"/>
       <c r="E24" s="5"/>
       <c r="F24" s="5"/>
       <c r="G24" s="6" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="25" spans="3:7" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+      <c r="H24" s="5"/>
+      <c r="I24" s="5"/>
+    </row>
+    <row r="25" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C25" s="5"/>
       <c r="D25" s="5"/>
       <c r="E25" s="5"/>
       <c r="F25" s="5"/>
       <c r="G25" s="6" t="s">
-        <v>22</v>
-      </c>
+        <v>20</v>
+      </c>
+      <c r="H25" s="5"/>
+      <c r="I25" s="5"/>
     </row>
   </sheetData>
-  <mergeCells count="24">
+  <mergeCells count="38">
+    <mergeCell ref="C4:C13"/>
+    <mergeCell ref="H14:H16"/>
+    <mergeCell ref="H17:H19"/>
+    <mergeCell ref="H20:H22"/>
+    <mergeCell ref="H23:H25"/>
+    <mergeCell ref="I14:I16"/>
+    <mergeCell ref="I17:I19"/>
+    <mergeCell ref="I20:I22"/>
+    <mergeCell ref="I23:I25"/>
+    <mergeCell ref="H4:H6"/>
+    <mergeCell ref="I4:I6"/>
+    <mergeCell ref="H7:H9"/>
+    <mergeCell ref="I7:I9"/>
+    <mergeCell ref="H10:H12"/>
+    <mergeCell ref="I10:I12"/>
     <mergeCell ref="E17:E19"/>
     <mergeCell ref="F17:F19"/>
     <mergeCell ref="D20:D22"/>
     <mergeCell ref="E20:E22"/>
     <mergeCell ref="F20:F22"/>
-    <mergeCell ref="C4:C13"/>
+    <mergeCell ref="D7:D9"/>
+    <mergeCell ref="E7:E9"/>
+    <mergeCell ref="F7:F9"/>
     <mergeCell ref="D4:D6"/>
     <mergeCell ref="E4:E6"/>
     <mergeCell ref="F4:F6"/>
-    <mergeCell ref="F8:F10"/>
-    <mergeCell ref="E8:E10"/>
-    <mergeCell ref="D11:D13"/>
-    <mergeCell ref="E11:E13"/>
-    <mergeCell ref="F11:F13"/>
+    <mergeCell ref="F10:F12"/>
+    <mergeCell ref="E10:E12"/>
     <mergeCell ref="F23:F25"/>
     <mergeCell ref="E23:E25"/>
     <mergeCell ref="D23:D25"/>
     <mergeCell ref="C23:C25"/>
     <mergeCell ref="C14:C22"/>
-    <mergeCell ref="D8:D10"/>
+    <mergeCell ref="D10:D12"/>
     <mergeCell ref="D14:D16"/>
     <mergeCell ref="E14:E16"/>
     <mergeCell ref="F14:F16"/>
     <mergeCell ref="D17:D19"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup scale="72" orientation="landscape" r:id="rId1"/>
+  <pageSetup scale="55" orientation="landscape" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add service delete use case
</commit_message>
<xml_diff>
--- a/docs/Methods.xlsx
+++ b/docs/Methods.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\API\ConferenceRoomBooking\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80672433-3294-4EDE-973C-36CEA4013C57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8279A587-3EC5-4B7B-A445-FB3D6BAB5104}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="4185" windowWidth="29040" windowHeight="15720" xr2:uid="{290D68D7-7384-40BB-827B-CD27B026537C}"/>
   </bookViews>
@@ -240,13 +240,7 @@
   </cellStyleXfs>
   <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -259,13 +253,19 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -622,126 +622,126 @@
       </c>
     </row>
     <row r="4" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="D4" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="E4" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="F4" s="5" t="s">
+      <c r="F4" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="G4" s="6" t="s">
+      <c r="G4" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="H4" s="5"/>
-      <c r="I4" s="5"/>
+      <c r="H4" s="8"/>
+      <c r="I4" s="8"/>
     </row>
     <row r="5" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C5" s="4"/>
-      <c r="D5" s="5"/>
-      <c r="E5" s="5"/>
-      <c r="F5" s="5"/>
-      <c r="G5" s="6" t="s">
+      <c r="C5" s="7"/>
+      <c r="D5" s="8"/>
+      <c r="E5" s="8"/>
+      <c r="F5" s="8"/>
+      <c r="G5" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="H5" s="5"/>
-      <c r="I5" s="5"/>
+      <c r="H5" s="8"/>
+      <c r="I5" s="8"/>
     </row>
     <row r="6" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C6" s="4"/>
-      <c r="D6" s="5"/>
-      <c r="E6" s="5"/>
-      <c r="F6" s="5"/>
-      <c r="G6" s="6" t="s">
+      <c r="C6" s="7"/>
+      <c r="D6" s="8"/>
+      <c r="E6" s="8"/>
+      <c r="F6" s="8"/>
+      <c r="G6" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="H6" s="5"/>
-      <c r="I6" s="5"/>
+      <c r="H6" s="8"/>
+      <c r="I6" s="8"/>
     </row>
     <row r="7" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C7" s="4"/>
-      <c r="D7" s="5" t="s">
+      <c r="C7" s="7"/>
+      <c r="D7" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="E7" s="5" t="s">
+      <c r="E7" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="F7" s="5" t="s">
+      <c r="F7" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="G7" s="6" t="s">
+      <c r="G7" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="H7" s="5"/>
-      <c r="I7" s="5"/>
+      <c r="H7" s="8"/>
+      <c r="I7" s="8"/>
     </row>
     <row r="8" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C8" s="4"/>
-      <c r="D8" s="5"/>
-      <c r="E8" s="5"/>
-      <c r="F8" s="5"/>
-      <c r="G8" s="6" t="s">
+      <c r="C8" s="7"/>
+      <c r="D8" s="8"/>
+      <c r="E8" s="8"/>
+      <c r="F8" s="8"/>
+      <c r="G8" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="H8" s="5"/>
-      <c r="I8" s="5"/>
+      <c r="H8" s="8"/>
+      <c r="I8" s="8"/>
     </row>
     <row r="9" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C9" s="4"/>
-      <c r="D9" s="5"/>
-      <c r="E9" s="5"/>
-      <c r="F9" s="5"/>
-      <c r="G9" s="6" t="s">
+      <c r="C9" s="7"/>
+      <c r="D9" s="8"/>
+      <c r="E9" s="8"/>
+      <c r="F9" s="8"/>
+      <c r="G9" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="H9" s="5"/>
-      <c r="I9" s="5"/>
+      <c r="H9" s="8"/>
+      <c r="I9" s="8"/>
     </row>
     <row r="10" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C10" s="4"/>
-      <c r="D10" s="5" t="s">
+      <c r="C10" s="7"/>
+      <c r="D10" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="E10" s="5" t="s">
+      <c r="E10" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="F10" s="5" t="s">
+      <c r="F10" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="G10" s="6" t="s">
+      <c r="G10" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="H10" s="5"/>
-      <c r="I10" s="5"/>
+      <c r="H10" s="8"/>
+      <c r="I10" s="8"/>
     </row>
     <row r="11" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C11" s="4"/>
-      <c r="D11" s="5"/>
-      <c r="E11" s="5"/>
-      <c r="F11" s="5"/>
-      <c r="G11" s="6" t="s">
+      <c r="C11" s="7"/>
+      <c r="D11" s="8"/>
+      <c r="E11" s="8"/>
+      <c r="F11" s="8"/>
+      <c r="G11" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="H11" s="5"/>
-      <c r="I11" s="5"/>
+      <c r="H11" s="8"/>
+      <c r="I11" s="8"/>
     </row>
     <row r="12" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C12" s="4"/>
-      <c r="D12" s="5"/>
-      <c r="E12" s="5"/>
-      <c r="F12" s="5"/>
-      <c r="G12" s="6" t="s">
+      <c r="C12" s="7"/>
+      <c r="D12" s="8"/>
+      <c r="E12" s="8"/>
+      <c r="F12" s="8"/>
+      <c r="G12" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="H12" s="5"/>
-      <c r="I12" s="5"/>
+      <c r="H12" s="8"/>
+      <c r="I12" s="8"/>
     </row>
     <row r="13" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C13" s="4"/>
+      <c r="C13" s="7"/>
       <c r="D13" s="3" t="s">
         <v>15</v>
       </c>
@@ -758,184 +758,191 @@
       <c r="I13" s="3"/>
     </row>
     <row r="14" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C14" s="5" t="s">
+      <c r="C14" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="D14" s="7" t="s">
+      <c r="D14" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="E14" s="7" t="s">
+      <c r="E14" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="F14" s="7" t="s">
+      <c r="F14" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="G14" s="8" t="s">
+      <c r="G14" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="H14" s="5" t="s">
+      <c r="H14" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="I14" s="5" t="s">
+      <c r="I14" s="9" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="15" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C15" s="5"/>
-      <c r="D15" s="7"/>
-      <c r="E15" s="7"/>
-      <c r="F15" s="7"/>
-      <c r="G15" s="8" t="s">
+      <c r="C15" s="9"/>
+      <c r="D15" s="9"/>
+      <c r="E15" s="9"/>
+      <c r="F15" s="9"/>
+      <c r="G15" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="H15" s="5"/>
-      <c r="I15" s="5"/>
+      <c r="H15" s="9"/>
+      <c r="I15" s="9"/>
     </row>
     <row r="16" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C16" s="5"/>
-      <c r="D16" s="7"/>
-      <c r="E16" s="7"/>
-      <c r="F16" s="7"/>
-      <c r="G16" s="8" t="s">
+      <c r="C16" s="9"/>
+      <c r="D16" s="9"/>
+      <c r="E16" s="9"/>
+      <c r="F16" s="9"/>
+      <c r="G16" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="H16" s="5"/>
-      <c r="I16" s="5"/>
+      <c r="H16" s="9"/>
+      <c r="I16" s="9"/>
     </row>
     <row r="17" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C17" s="5"/>
-      <c r="D17" s="7" t="s">
+      <c r="C17" s="9"/>
+      <c r="D17" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="E17" s="7" t="s">
+      <c r="E17" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="F17" s="7" t="s">
+      <c r="F17" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="G17" s="8" t="s">
+      <c r="G17" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="H17" s="5" t="s">
+      <c r="H17" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="I17" s="5" t="s">
+      <c r="I17" s="9" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="18" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C18" s="5"/>
-      <c r="D18" s="7"/>
-      <c r="E18" s="7"/>
-      <c r="F18" s="7"/>
-      <c r="G18" s="9" t="s">
+      <c r="C18" s="9"/>
+      <c r="D18" s="9"/>
+      <c r="E18" s="9"/>
+      <c r="F18" s="9"/>
+      <c r="G18" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="H18" s="5"/>
-      <c r="I18" s="5"/>
+      <c r="H18" s="9"/>
+      <c r="I18" s="9"/>
     </row>
     <row r="19" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C19" s="5"/>
-      <c r="D19" s="7"/>
-      <c r="E19" s="7"/>
-      <c r="F19" s="7"/>
-      <c r="G19" s="9" t="s">
+      <c r="C19" s="9"/>
+      <c r="D19" s="9"/>
+      <c r="E19" s="9"/>
+      <c r="F19" s="9"/>
+      <c r="G19" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="H19" s="5"/>
-      <c r="I19" s="5"/>
+      <c r="H19" s="9"/>
+      <c r="I19" s="9"/>
     </row>
     <row r="20" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C20" s="5"/>
-      <c r="D20" s="5" t="s">
+      <c r="C20" s="9"/>
+      <c r="D20" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="E20" s="5" t="s">
+      <c r="E20" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="F20" s="5" t="s">
+      <c r="F20" s="9" t="s">
         <v>25</v>
       </c>
       <c r="G20" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="H20" s="5" t="s">
+      <c r="H20" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="I20" s="5" t="s">
+      <c r="I20" s="9" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="21" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C21" s="5"/>
-      <c r="D21" s="5"/>
-      <c r="E21" s="5"/>
-      <c r="F21" s="5"/>
-      <c r="G21" s="6" t="s">
+      <c r="C21" s="9"/>
+      <c r="D21" s="9"/>
+      <c r="E21" s="9"/>
+      <c r="F21" s="9"/>
+      <c r="G21" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="H21" s="5"/>
-      <c r="I21" s="5"/>
+      <c r="H21" s="9"/>
+      <c r="I21" s="9"/>
     </row>
     <row r="22" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C22" s="5"/>
-      <c r="D22" s="5"/>
-      <c r="E22" s="5"/>
-      <c r="F22" s="5"/>
+      <c r="C22" s="9"/>
+      <c r="D22" s="9"/>
+      <c r="E22" s="9"/>
+      <c r="F22" s="9"/>
       <c r="G22" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="H22" s="5"/>
-      <c r="I22" s="5"/>
+      <c r="H22" s="9"/>
+      <c r="I22" s="9"/>
     </row>
     <row r="23" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C23" s="5" t="s">
+      <c r="C23" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="D23" s="5" t="s">
+      <c r="D23" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="E23" s="5" t="s">
+      <c r="E23" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="F23" s="5" t="s">
+      <c r="F23" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="G23" s="6" t="s">
+      <c r="G23" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="H23" s="5"/>
-      <c r="I23" s="5"/>
+      <c r="H23" s="8"/>
+      <c r="I23" s="8"/>
     </row>
     <row r="24" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C24" s="5"/>
-      <c r="D24" s="5"/>
-      <c r="E24" s="5"/>
-      <c r="F24" s="5"/>
-      <c r="G24" s="6" t="s">
+      <c r="C24" s="8"/>
+      <c r="D24" s="8"/>
+      <c r="E24" s="8"/>
+      <c r="F24" s="8"/>
+      <c r="G24" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="H24" s="5"/>
-      <c r="I24" s="5"/>
+      <c r="H24" s="8"/>
+      <c r="I24" s="8"/>
     </row>
     <row r="25" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C25" s="5"/>
-      <c r="D25" s="5"/>
-      <c r="E25" s="5"/>
-      <c r="F25" s="5"/>
-      <c r="G25" s="6" t="s">
+      <c r="C25" s="8"/>
+      <c r="D25" s="8"/>
+      <c r="E25" s="8"/>
+      <c r="F25" s="8"/>
+      <c r="G25" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="H25" s="5"/>
-      <c r="I25" s="5"/>
+      <c r="H25" s="8"/>
+      <c r="I25" s="8"/>
     </row>
   </sheetData>
   <mergeCells count="38">
-    <mergeCell ref="C4:C13"/>
-    <mergeCell ref="H14:H16"/>
-    <mergeCell ref="H17:H19"/>
-    <mergeCell ref="H20:H22"/>
-    <mergeCell ref="H23:H25"/>
+    <mergeCell ref="C23:C25"/>
+    <mergeCell ref="C14:C22"/>
+    <mergeCell ref="D10:D12"/>
+    <mergeCell ref="D14:D16"/>
+    <mergeCell ref="E14:E16"/>
+    <mergeCell ref="D17:D19"/>
+    <mergeCell ref="F10:F12"/>
+    <mergeCell ref="E10:E12"/>
+    <mergeCell ref="F23:F25"/>
+    <mergeCell ref="E23:E25"/>
+    <mergeCell ref="D23:D25"/>
+    <mergeCell ref="F14:F16"/>
     <mergeCell ref="I14:I16"/>
     <mergeCell ref="I17:I19"/>
     <mergeCell ref="I20:I22"/>
@@ -946,6 +953,11 @@
     <mergeCell ref="I7:I9"/>
     <mergeCell ref="H10:H12"/>
     <mergeCell ref="I10:I12"/>
+    <mergeCell ref="C4:C13"/>
+    <mergeCell ref="H14:H16"/>
+    <mergeCell ref="H17:H19"/>
+    <mergeCell ref="H20:H22"/>
+    <mergeCell ref="H23:H25"/>
     <mergeCell ref="E17:E19"/>
     <mergeCell ref="F17:F19"/>
     <mergeCell ref="D20:D22"/>
@@ -957,18 +969,6 @@
     <mergeCell ref="D4:D6"/>
     <mergeCell ref="E4:E6"/>
     <mergeCell ref="F4:F6"/>
-    <mergeCell ref="F10:F12"/>
-    <mergeCell ref="E10:E12"/>
-    <mergeCell ref="F23:F25"/>
-    <mergeCell ref="E23:E25"/>
-    <mergeCell ref="D23:D25"/>
-    <mergeCell ref="C23:C25"/>
-    <mergeCell ref="C14:C22"/>
-    <mergeCell ref="D10:D12"/>
-    <mergeCell ref="D14:D16"/>
-    <mergeCell ref="E14:E16"/>
-    <mergeCell ref="F14:F16"/>
-    <mergeCell ref="D17:D19"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup scale="55" orientation="landscape" r:id="rId1"/>

</xml_diff>

<commit_message>
Add conference room create use case
</commit_message>
<xml_diff>
--- a/docs/Methods.xlsx
+++ b/docs/Methods.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\API\ConferenceRoomBooking\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8279A587-3EC5-4B7B-A445-FB3D6BAB5104}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1380EAED-3878-40CC-8D3A-033A739F50FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="4185" windowWidth="29040" windowHeight="15720" xr2:uid="{290D68D7-7384-40BB-827B-CD27B026537C}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="47">
   <si>
     <t>Method</t>
   </si>
@@ -163,6 +163,18 @@
   </si>
   <si>
     <t>Application Service</t>
+  </si>
+  <si>
+    <t>POST /api/conference-rooms</t>
+  </si>
+  <si>
+    <t>PUT /api/conference-rooms/{id}</t>
+  </si>
+  <si>
+    <t>DELETE /api/conference-rooms/{id}</t>
+  </si>
+  <si>
+    <t>GetByIdWithServicesAsync()</t>
   </si>
 </sst>
 </file>
@@ -258,13 +270,13 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -594,7 +606,7 @@
     <col min="6" max="6" width="52.140625" style="1" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="34.85546875" style="1" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="19.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="28.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="36" style="1" bestFit="1" customWidth="1"/>
     <col min="10" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
@@ -622,7 +634,7 @@
       </c>
     </row>
     <row r="4" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C4" s="7" t="s">
+      <c r="C4" s="9" t="s">
         <v>4</v>
       </c>
       <c r="D4" s="8" t="s">
@@ -634,114 +646,126 @@
       <c r="F4" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="G4" s="4" t="s">
+      <c r="G4" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="H4" s="8"/>
-      <c r="I4" s="8"/>
+      <c r="H4" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="I4" s="8" t="s">
+        <v>43</v>
+      </c>
     </row>
     <row r="5" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C5" s="7"/>
+      <c r="C5" s="9"/>
       <c r="D5" s="8"/>
       <c r="E5" s="8"/>
       <c r="F5" s="8"/>
-      <c r="G5" s="4" t="s">
+      <c r="G5" s="5" t="s">
         <v>9</v>
       </c>
       <c r="H5" s="8"/>
       <c r="I5" s="8"/>
     </row>
     <row r="6" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C6" s="7"/>
+      <c r="C6" s="9"/>
       <c r="D6" s="8"/>
       <c r="E6" s="8"/>
       <c r="F6" s="8"/>
-      <c r="G6" s="4" t="s">
+      <c r="G6" s="5" t="s">
         <v>10</v>
       </c>
       <c r="H6" s="8"/>
       <c r="I6" s="8"/>
     </row>
     <row r="7" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C7" s="7"/>
-      <c r="D7" s="8" t="s">
+      <c r="C7" s="9"/>
+      <c r="D7" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="E7" s="8" t="s">
+      <c r="E7" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="F7" s="8" t="s">
+      <c r="F7" s="7" t="s">
         <v>22</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="H7" s="8"/>
-      <c r="I7" s="8"/>
+        <v>46</v>
+      </c>
+      <c r="H7" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="I7" s="7" t="s">
+        <v>44</v>
+      </c>
     </row>
     <row r="8" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C8" s="7"/>
-      <c r="D8" s="8"/>
-      <c r="E8" s="8"/>
-      <c r="F8" s="8"/>
+      <c r="C8" s="9"/>
+      <c r="D8" s="7"/>
+      <c r="E8" s="7"/>
+      <c r="F8" s="7"/>
       <c r="G8" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="H8" s="8"/>
-      <c r="I8" s="8"/>
+      <c r="H8" s="7"/>
+      <c r="I8" s="7"/>
     </row>
     <row r="9" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C9" s="7"/>
-      <c r="D9" s="8"/>
-      <c r="E9" s="8"/>
-      <c r="F9" s="8"/>
+      <c r="C9" s="9"/>
+      <c r="D9" s="7"/>
+      <c r="E9" s="7"/>
+      <c r="F9" s="7"/>
       <c r="G9" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="H9" s="8"/>
-      <c r="I9" s="8"/>
+      <c r="H9" s="7"/>
+      <c r="I9" s="7"/>
     </row>
     <row r="10" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C10" s="7"/>
-      <c r="D10" s="8" t="s">
+      <c r="C10" s="9"/>
+      <c r="D10" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="E10" s="8" t="s">
+      <c r="E10" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="F10" s="8" t="s">
+      <c r="F10" s="7" t="s">
         <v>22</v>
       </c>
       <c r="G10" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="H10" s="8"/>
-      <c r="I10" s="8"/>
+      <c r="H10" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="I10" s="7" t="s">
+        <v>45</v>
+      </c>
     </row>
     <row r="11" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C11" s="7"/>
-      <c r="D11" s="8"/>
-      <c r="E11" s="8"/>
-      <c r="F11" s="8"/>
+      <c r="C11" s="9"/>
+      <c r="D11" s="7"/>
+      <c r="E11" s="7"/>
+      <c r="F11" s="7"/>
       <c r="G11" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="H11" s="8"/>
-      <c r="I11" s="8"/>
+      <c r="H11" s="7"/>
+      <c r="I11" s="7"/>
     </row>
     <row r="12" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C12" s="7"/>
-      <c r="D12" s="8"/>
-      <c r="E12" s="8"/>
-      <c r="F12" s="8"/>
+      <c r="C12" s="9"/>
+      <c r="D12" s="7"/>
+      <c r="E12" s="7"/>
+      <c r="F12" s="7"/>
       <c r="G12" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="H12" s="8"/>
-      <c r="I12" s="8"/>
+      <c r="H12" s="7"/>
+      <c r="I12" s="7"/>
     </row>
     <row r="13" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C13" s="7"/>
+      <c r="C13" s="9"/>
       <c r="D13" s="3" t="s">
         <v>15</v>
       </c>
@@ -758,191 +782,183 @@
       <c r="I13" s="3"/>
     </row>
     <row r="14" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C14" s="9" t="s">
+      <c r="C14" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="D14" s="9" t="s">
+      <c r="D14" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="E14" s="9" t="s">
+      <c r="E14" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="F14" s="9" t="s">
+      <c r="F14" s="8" t="s">
         <v>24</v>
       </c>
       <c r="G14" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="H14" s="9" t="s">
+      <c r="H14" s="8" t="s">
         <v>36</v>
       </c>
-      <c r="I14" s="9" t="s">
+      <c r="I14" s="8" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="15" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C15" s="9"/>
-      <c r="D15" s="9"/>
-      <c r="E15" s="9"/>
-      <c r="F15" s="9"/>
+      <c r="C15" s="8"/>
+      <c r="D15" s="8"/>
+      <c r="E15" s="8"/>
+      <c r="F15" s="8"/>
       <c r="G15" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="H15" s="9"/>
-      <c r="I15" s="9"/>
+      <c r="H15" s="8"/>
+      <c r="I15" s="8"/>
     </row>
     <row r="16" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C16" s="9"/>
-      <c r="D16" s="9"/>
-      <c r="E16" s="9"/>
-      <c r="F16" s="9"/>
+      <c r="C16" s="8"/>
+      <c r="D16" s="8"/>
+      <c r="E16" s="8"/>
+      <c r="F16" s="8"/>
       <c r="G16" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="H16" s="9"/>
-      <c r="I16" s="9"/>
+      <c r="H16" s="8"/>
+      <c r="I16" s="8"/>
     </row>
     <row r="17" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C17" s="9"/>
-      <c r="D17" s="9" t="s">
+      <c r="C17" s="8"/>
+      <c r="D17" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="E17" s="9" t="s">
+      <c r="E17" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="F17" s="9" t="s">
+      <c r="F17" s="8" t="s">
         <v>25</v>
       </c>
       <c r="G17" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="H17" s="9" t="s">
+      <c r="H17" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="I17" s="9" t="s">
+      <c r="I17" s="8" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="18" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C18" s="9"/>
-      <c r="D18" s="9"/>
-      <c r="E18" s="9"/>
-      <c r="F18" s="9"/>
+      <c r="C18" s="8"/>
+      <c r="D18" s="8"/>
+      <c r="E18" s="8"/>
+      <c r="F18" s="8"/>
       <c r="G18" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="H18" s="9"/>
-      <c r="I18" s="9"/>
+      <c r="H18" s="8"/>
+      <c r="I18" s="8"/>
     </row>
     <row r="19" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C19" s="9"/>
-      <c r="D19" s="9"/>
-      <c r="E19" s="9"/>
-      <c r="F19" s="9"/>
+      <c r="C19" s="8"/>
+      <c r="D19" s="8"/>
+      <c r="E19" s="8"/>
+      <c r="F19" s="8"/>
       <c r="G19" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="H19" s="9"/>
-      <c r="I19" s="9"/>
+      <c r="H19" s="8"/>
+      <c r="I19" s="8"/>
     </row>
     <row r="20" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C20" s="9"/>
-      <c r="D20" s="9" t="s">
+      <c r="C20" s="8"/>
+      <c r="D20" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="E20" s="9" t="s">
+      <c r="E20" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="F20" s="9" t="s">
+      <c r="F20" s="8" t="s">
         <v>25</v>
       </c>
       <c r="G20" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="H20" s="9" t="s">
+      <c r="H20" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="I20" s="9" t="s">
+      <c r="I20" s="8" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="21" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C21" s="9"/>
-      <c r="D21" s="9"/>
-      <c r="E21" s="9"/>
-      <c r="F21" s="9"/>
+      <c r="C21" s="8"/>
+      <c r="D21" s="8"/>
+      <c r="E21" s="8"/>
+      <c r="F21" s="8"/>
       <c r="G21" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="H21" s="9"/>
-      <c r="I21" s="9"/>
+      <c r="H21" s="8"/>
+      <c r="I21" s="8"/>
     </row>
     <row r="22" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C22" s="9"/>
-      <c r="D22" s="9"/>
-      <c r="E22" s="9"/>
-      <c r="F22" s="9"/>
+      <c r="C22" s="8"/>
+      <c r="D22" s="8"/>
+      <c r="E22" s="8"/>
+      <c r="F22" s="8"/>
       <c r="G22" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="H22" s="9"/>
-      <c r="I22" s="9"/>
+      <c r="H22" s="8"/>
+      <c r="I22" s="8"/>
     </row>
     <row r="23" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C23" s="8" t="s">
+      <c r="C23" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="D23" s="8" t="s">
+      <c r="D23" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="E23" s="8" t="s">
+      <c r="E23" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="F23" s="8" t="s">
+      <c r="F23" s="7" t="s">
         <v>26</v>
       </c>
       <c r="G23" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="H23" s="8"/>
-      <c r="I23" s="8"/>
+      <c r="H23" s="7"/>
+      <c r="I23" s="7"/>
     </row>
     <row r="24" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C24" s="8"/>
-      <c r="D24" s="8"/>
-      <c r="E24" s="8"/>
-      <c r="F24" s="8"/>
+      <c r="C24" s="7"/>
+      <c r="D24" s="7"/>
+      <c r="E24" s="7"/>
+      <c r="F24" s="7"/>
       <c r="G24" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="H24" s="8"/>
-      <c r="I24" s="8"/>
+      <c r="H24" s="7"/>
+      <c r="I24" s="7"/>
     </row>
     <row r="25" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C25" s="8"/>
-      <c r="D25" s="8"/>
-      <c r="E25" s="8"/>
-      <c r="F25" s="8"/>
+      <c r="C25" s="7"/>
+      <c r="D25" s="7"/>
+      <c r="E25" s="7"/>
+      <c r="F25" s="7"/>
       <c r="G25" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="H25" s="8"/>
-      <c r="I25" s="8"/>
+      <c r="H25" s="7"/>
+      <c r="I25" s="7"/>
     </row>
   </sheetData>
   <mergeCells count="38">
-    <mergeCell ref="C23:C25"/>
-    <mergeCell ref="C14:C22"/>
-    <mergeCell ref="D10:D12"/>
-    <mergeCell ref="D14:D16"/>
-    <mergeCell ref="E14:E16"/>
-    <mergeCell ref="D17:D19"/>
-    <mergeCell ref="F10:F12"/>
-    <mergeCell ref="E10:E12"/>
-    <mergeCell ref="F23:F25"/>
-    <mergeCell ref="E23:E25"/>
-    <mergeCell ref="D23:D25"/>
-    <mergeCell ref="F14:F16"/>
+    <mergeCell ref="F7:F9"/>
+    <mergeCell ref="D4:D6"/>
+    <mergeCell ref="E4:E6"/>
+    <mergeCell ref="F4:F6"/>
     <mergeCell ref="I14:I16"/>
     <mergeCell ref="I17:I19"/>
     <mergeCell ref="I20:I22"/>
@@ -953,22 +969,30 @@
     <mergeCell ref="I7:I9"/>
     <mergeCell ref="H10:H12"/>
     <mergeCell ref="I10:I12"/>
-    <mergeCell ref="C4:C13"/>
     <mergeCell ref="H14:H16"/>
     <mergeCell ref="H17:H19"/>
     <mergeCell ref="H20:H22"/>
     <mergeCell ref="H23:H25"/>
+    <mergeCell ref="F10:F12"/>
+    <mergeCell ref="E10:E12"/>
+    <mergeCell ref="F23:F25"/>
+    <mergeCell ref="E23:E25"/>
+    <mergeCell ref="D23:D25"/>
+    <mergeCell ref="F14:F16"/>
     <mergeCell ref="E17:E19"/>
     <mergeCell ref="F17:F19"/>
     <mergeCell ref="D20:D22"/>
     <mergeCell ref="E20:E22"/>
     <mergeCell ref="F20:F22"/>
+    <mergeCell ref="C23:C25"/>
+    <mergeCell ref="C14:C22"/>
+    <mergeCell ref="D10:D12"/>
+    <mergeCell ref="D14:D16"/>
+    <mergeCell ref="E14:E16"/>
+    <mergeCell ref="D17:D19"/>
+    <mergeCell ref="C4:C13"/>
     <mergeCell ref="D7:D9"/>
     <mergeCell ref="E7:E9"/>
-    <mergeCell ref="F7:F9"/>
-    <mergeCell ref="D4:D6"/>
-    <mergeCell ref="E4:E6"/>
-    <mergeCell ref="F4:F6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup scale="55" orientation="landscape" r:id="rId1"/>

</xml_diff>

<commit_message>
Add conference room update use case
</commit_message>
<xml_diff>
--- a/docs/Methods.xlsx
+++ b/docs/Methods.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\API\ConferenceRoomBooking\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1380EAED-3878-40CC-8D3A-033A739F50FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1514C979-5D3C-4565-979B-1FE50ACD9355}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="4185" windowWidth="29040" windowHeight="15720" xr2:uid="{290D68D7-7384-40BB-827B-CD27B026537C}"/>
   </bookViews>
@@ -680,46 +680,46 @@
     </row>
     <row r="7" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C7" s="9"/>
-      <c r="D7" s="7" t="s">
+      <c r="D7" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="E7" s="7" t="s">
+      <c r="E7" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="F7" s="7" t="s">
+      <c r="F7" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="G7" s="4" t="s">
+      <c r="G7" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="H7" s="7" t="s">
+      <c r="H7" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="I7" s="7" t="s">
+      <c r="I7" s="8" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="8" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C8" s="9"/>
-      <c r="D8" s="7"/>
-      <c r="E8" s="7"/>
-      <c r="F8" s="7"/>
-      <c r="G8" s="4" t="s">
+      <c r="D8" s="8"/>
+      <c r="E8" s="8"/>
+      <c r="F8" s="8"/>
+      <c r="G8" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="H8" s="7"/>
-      <c r="I8" s="7"/>
+      <c r="H8" s="8"/>
+      <c r="I8" s="8"/>
     </row>
     <row r="9" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C9" s="9"/>
-      <c r="D9" s="7"/>
-      <c r="E9" s="7"/>
-      <c r="F9" s="7"/>
-      <c r="G9" s="4" t="s">
+      <c r="D9" s="8"/>
+      <c r="E9" s="8"/>
+      <c r="F9" s="8"/>
+      <c r="G9" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="H9" s="7"/>
-      <c r="I9" s="7"/>
+      <c r="H9" s="8"/>
+      <c r="I9" s="8"/>
     </row>
     <row r="10" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C10" s="9"/>
@@ -955,11 +955,24 @@
     </row>
   </sheetData>
   <mergeCells count="38">
-    <mergeCell ref="F7:F9"/>
-    <mergeCell ref="D4:D6"/>
-    <mergeCell ref="E4:E6"/>
-    <mergeCell ref="F4:F6"/>
-    <mergeCell ref="I14:I16"/>
+    <mergeCell ref="C23:C25"/>
+    <mergeCell ref="C14:C22"/>
+    <mergeCell ref="D10:D12"/>
+    <mergeCell ref="D14:D16"/>
+    <mergeCell ref="E14:E16"/>
+    <mergeCell ref="D17:D19"/>
+    <mergeCell ref="C4:C13"/>
+    <mergeCell ref="D7:D9"/>
+    <mergeCell ref="E7:E9"/>
+    <mergeCell ref="F23:F25"/>
+    <mergeCell ref="E23:E25"/>
+    <mergeCell ref="D23:D25"/>
+    <mergeCell ref="F14:F16"/>
+    <mergeCell ref="E17:E19"/>
+    <mergeCell ref="F17:F19"/>
+    <mergeCell ref="D20:D22"/>
+    <mergeCell ref="E20:E22"/>
+    <mergeCell ref="F20:F22"/>
     <mergeCell ref="I17:I19"/>
     <mergeCell ref="I20:I22"/>
     <mergeCell ref="I23:I25"/>
@@ -973,26 +986,13 @@
     <mergeCell ref="H17:H19"/>
     <mergeCell ref="H20:H22"/>
     <mergeCell ref="H23:H25"/>
+    <mergeCell ref="F7:F9"/>
+    <mergeCell ref="D4:D6"/>
+    <mergeCell ref="E4:E6"/>
+    <mergeCell ref="F4:F6"/>
+    <mergeCell ref="I14:I16"/>
     <mergeCell ref="F10:F12"/>
     <mergeCell ref="E10:E12"/>
-    <mergeCell ref="F23:F25"/>
-    <mergeCell ref="E23:E25"/>
-    <mergeCell ref="D23:D25"/>
-    <mergeCell ref="F14:F16"/>
-    <mergeCell ref="E17:E19"/>
-    <mergeCell ref="F17:F19"/>
-    <mergeCell ref="D20:D22"/>
-    <mergeCell ref="E20:E22"/>
-    <mergeCell ref="F20:F22"/>
-    <mergeCell ref="C23:C25"/>
-    <mergeCell ref="C14:C22"/>
-    <mergeCell ref="D10:D12"/>
-    <mergeCell ref="D14:D16"/>
-    <mergeCell ref="E14:E16"/>
-    <mergeCell ref="D17:D19"/>
-    <mergeCell ref="C4:C13"/>
-    <mergeCell ref="D7:D9"/>
-    <mergeCell ref="E7:E9"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup scale="55" orientation="landscape" r:id="rId1"/>

</xml_diff>

<commit_message>
Add conference room Search Available use case
</commit_message>
<xml_diff>
--- a/docs/Methods.xlsx
+++ b/docs/Methods.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\API\ConferenceRoomBooking\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1514C979-5D3C-4565-979B-1FE50ACD9355}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F660ECCF-40BB-4EA8-A329-857B7DD370B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="4185" windowWidth="29040" windowHeight="15720" xr2:uid="{290D68D7-7384-40BB-827B-CD27B026537C}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="49">
   <si>
     <t>Method</t>
   </si>
@@ -175,6 +175,12 @@
   </si>
   <si>
     <t>GetByIdWithServicesAsync()</t>
+  </si>
+  <si>
+    <t>SearchAvailable</t>
+  </si>
+  <si>
+    <t>POST /api/conference-rooms/search</t>
   </si>
 </sst>
 </file>
@@ -250,7 +256,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -269,6 +275,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -634,345 +643,338 @@
       </c>
     </row>
     <row r="4" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C4" s="9" t="s">
+      <c r="C4" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="D4" s="8" t="s">
+      <c r="D4" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="8" t="s">
+      <c r="E4" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="F4" s="8" t="s">
+      <c r="F4" s="9" t="s">
         <v>7</v>
       </c>
       <c r="G4" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="H4" s="8" t="s">
+      <c r="H4" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="I4" s="8" t="s">
+      <c r="I4" s="9" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="5" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C5" s="9"/>
-      <c r="D5" s="8"/>
-      <c r="E5" s="8"/>
-      <c r="F5" s="8"/>
+      <c r="C5" s="10"/>
+      <c r="D5" s="9"/>
+      <c r="E5" s="9"/>
+      <c r="F5" s="9"/>
       <c r="G5" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="H5" s="8"/>
-      <c r="I5" s="8"/>
+      <c r="H5" s="9"/>
+      <c r="I5" s="9"/>
     </row>
     <row r="6" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C6" s="9"/>
-      <c r="D6" s="8"/>
-      <c r="E6" s="8"/>
-      <c r="F6" s="8"/>
+      <c r="C6" s="10"/>
+      <c r="D6" s="9"/>
+      <c r="E6" s="9"/>
+      <c r="F6" s="9"/>
       <c r="G6" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="H6" s="8"/>
-      <c r="I6" s="8"/>
+      <c r="H6" s="9"/>
+      <c r="I6" s="9"/>
     </row>
     <row r="7" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C7" s="9"/>
-      <c r="D7" s="8" t="s">
+      <c r="C7" s="10"/>
+      <c r="D7" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="E7" s="8" t="s">
+      <c r="E7" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="F7" s="8" t="s">
+      <c r="F7" s="9" t="s">
         <v>22</v>
       </c>
       <c r="G7" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="H7" s="8" t="s">
+      <c r="H7" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="I7" s="8" t="s">
+      <c r="I7" s="9" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="8" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C8" s="9"/>
-      <c r="D8" s="8"/>
-      <c r="E8" s="8"/>
-      <c r="F8" s="8"/>
+      <c r="C8" s="10"/>
+      <c r="D8" s="9"/>
+      <c r="E8" s="9"/>
+      <c r="F8" s="9"/>
       <c r="G8" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="H8" s="8"/>
-      <c r="I8" s="8"/>
+      <c r="H8" s="9"/>
+      <c r="I8" s="9"/>
     </row>
     <row r="9" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C9" s="9"/>
-      <c r="D9" s="8"/>
-      <c r="E9" s="8"/>
-      <c r="F9" s="8"/>
+      <c r="C9" s="10"/>
+      <c r="D9" s="9"/>
+      <c r="E9" s="9"/>
+      <c r="F9" s="9"/>
       <c r="G9" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="H9" s="8"/>
-      <c r="I9" s="8"/>
+      <c r="H9" s="9"/>
+      <c r="I9" s="9"/>
     </row>
     <row r="10" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C10" s="9"/>
-      <c r="D10" s="7" t="s">
+      <c r="C10" s="10"/>
+      <c r="D10" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="E10" s="7" t="s">
+      <c r="E10" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="F10" s="7" t="s">
+      <c r="F10" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="G10" s="4" t="s">
+      <c r="G10" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="H10" s="7" t="s">
+      <c r="H10" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="I10" s="7" t="s">
+      <c r="I10" s="9" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="11" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C11" s="9"/>
-      <c r="D11" s="7"/>
-      <c r="E11" s="7"/>
-      <c r="F11" s="7"/>
-      <c r="G11" s="4" t="s">
+      <c r="C11" s="10"/>
+      <c r="D11" s="9"/>
+      <c r="E11" s="9"/>
+      <c r="F11" s="9"/>
+      <c r="G11" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="H11" s="7"/>
-      <c r="I11" s="7"/>
+      <c r="H11" s="9"/>
+      <c r="I11" s="9"/>
     </row>
     <row r="12" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C12" s="9"/>
-      <c r="D12" s="7"/>
-      <c r="E12" s="7"/>
-      <c r="F12" s="7"/>
-      <c r="G12" s="4" t="s">
+      <c r="C12" s="10"/>
+      <c r="D12" s="9"/>
+      <c r="E12" s="9"/>
+      <c r="F12" s="9"/>
+      <c r="G12" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="H12" s="7"/>
-      <c r="I12" s="7"/>
+      <c r="H12" s="9"/>
+      <c r="I12" s="9"/>
     </row>
     <row r="13" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C13" s="9"/>
-      <c r="D13" s="3" t="s">
+      <c r="C13" s="10"/>
+      <c r="D13" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="E13" s="3" t="s">
+      <c r="E13" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="F13" s="3" t="s">
+      <c r="F13" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="G13" s="3" t="s">
+      <c r="G13" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="H13" s="3"/>
-      <c r="I13" s="3"/>
+      <c r="H13" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="I13" s="7" t="s">
+        <v>48</v>
+      </c>
     </row>
     <row r="14" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C14" s="8" t="s">
+      <c r="C14" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="D14" s="8" t="s">
+      <c r="D14" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="E14" s="8" t="s">
+      <c r="E14" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="F14" s="8" t="s">
+      <c r="F14" s="9" t="s">
         <v>24</v>
       </c>
       <c r="G14" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="H14" s="8" t="s">
+      <c r="H14" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="I14" s="8" t="s">
+      <c r="I14" s="9" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="15" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C15" s="8"/>
-      <c r="D15" s="8"/>
-      <c r="E15" s="8"/>
-      <c r="F15" s="8"/>
+      <c r="C15" s="9"/>
+      <c r="D15" s="9"/>
+      <c r="E15" s="9"/>
+      <c r="F15" s="9"/>
       <c r="G15" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="H15" s="8"/>
-      <c r="I15" s="8"/>
+      <c r="H15" s="9"/>
+      <c r="I15" s="9"/>
     </row>
     <row r="16" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C16" s="8"/>
-      <c r="D16" s="8"/>
-      <c r="E16" s="8"/>
-      <c r="F16" s="8"/>
+      <c r="C16" s="9"/>
+      <c r="D16" s="9"/>
+      <c r="E16" s="9"/>
+      <c r="F16" s="9"/>
       <c r="G16" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="H16" s="8"/>
-      <c r="I16" s="8"/>
+      <c r="H16" s="9"/>
+      <c r="I16" s="9"/>
     </row>
     <row r="17" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C17" s="8"/>
-      <c r="D17" s="8" t="s">
+      <c r="C17" s="9"/>
+      <c r="D17" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="E17" s="8" t="s">
+      <c r="E17" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="F17" s="8" t="s">
+      <c r="F17" s="9" t="s">
         <v>25</v>
       </c>
       <c r="G17" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="H17" s="8" t="s">
+      <c r="H17" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="I17" s="8" t="s">
+      <c r="I17" s="9" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="18" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C18" s="8"/>
-      <c r="D18" s="8"/>
-      <c r="E18" s="8"/>
-      <c r="F18" s="8"/>
+      <c r="C18" s="9"/>
+      <c r="D18" s="9"/>
+      <c r="E18" s="9"/>
+      <c r="F18" s="9"/>
       <c r="G18" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="H18" s="8"/>
-      <c r="I18" s="8"/>
+      <c r="H18" s="9"/>
+      <c r="I18" s="9"/>
     </row>
     <row r="19" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C19" s="8"/>
-      <c r="D19" s="8"/>
-      <c r="E19" s="8"/>
-      <c r="F19" s="8"/>
+      <c r="C19" s="9"/>
+      <c r="D19" s="9"/>
+      <c r="E19" s="9"/>
+      <c r="F19" s="9"/>
       <c r="G19" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="H19" s="8"/>
-      <c r="I19" s="8"/>
+      <c r="H19" s="9"/>
+      <c r="I19" s="9"/>
     </row>
     <row r="20" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C20" s="8"/>
-      <c r="D20" s="8" t="s">
+      <c r="C20" s="9"/>
+      <c r="D20" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="E20" s="8" t="s">
+      <c r="E20" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="F20" s="8" t="s">
+      <c r="F20" s="9" t="s">
         <v>25</v>
       </c>
       <c r="G20" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="H20" s="8" t="s">
+      <c r="H20" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="I20" s="8" t="s">
+      <c r="I20" s="9" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="21" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C21" s="8"/>
-      <c r="D21" s="8"/>
-      <c r="E21" s="8"/>
-      <c r="F21" s="8"/>
+      <c r="C21" s="9"/>
+      <c r="D21" s="9"/>
+      <c r="E21" s="9"/>
+      <c r="F21" s="9"/>
       <c r="G21" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="H21" s="8"/>
-      <c r="I21" s="8"/>
+      <c r="H21" s="9"/>
+      <c r="I21" s="9"/>
     </row>
     <row r="22" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C22" s="8"/>
-      <c r="D22" s="8"/>
-      <c r="E22" s="8"/>
-      <c r="F22" s="8"/>
+      <c r="C22" s="9"/>
+      <c r="D22" s="9"/>
+      <c r="E22" s="9"/>
+      <c r="F22" s="9"/>
       <c r="G22" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="H22" s="8"/>
-      <c r="I22" s="8"/>
+      <c r="H22" s="9"/>
+      <c r="I22" s="9"/>
     </row>
     <row r="23" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C23" s="7" t="s">
+      <c r="C23" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="D23" s="7" t="s">
+      <c r="D23" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="E23" s="7" t="s">
+      <c r="E23" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="F23" s="7" t="s">
+      <c r="F23" s="8" t="s">
         <v>26</v>
       </c>
       <c r="G23" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="H23" s="7"/>
-      <c r="I23" s="7"/>
+      <c r="H23" s="8"/>
+      <c r="I23" s="8"/>
     </row>
     <row r="24" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C24" s="7"/>
-      <c r="D24" s="7"/>
-      <c r="E24" s="7"/>
-      <c r="F24" s="7"/>
+      <c r="C24" s="8"/>
+      <c r="D24" s="8"/>
+      <c r="E24" s="8"/>
+      <c r="F24" s="8"/>
       <c r="G24" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="H24" s="7"/>
-      <c r="I24" s="7"/>
+      <c r="H24" s="8"/>
+      <c r="I24" s="8"/>
     </row>
     <row r="25" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C25" s="7"/>
-      <c r="D25" s="7"/>
-      <c r="E25" s="7"/>
-      <c r="F25" s="7"/>
+      <c r="C25" s="8"/>
+      <c r="D25" s="8"/>
+      <c r="E25" s="8"/>
+      <c r="F25" s="8"/>
       <c r="G25" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="H25" s="7"/>
-      <c r="I25" s="7"/>
+      <c r="H25" s="8"/>
+      <c r="I25" s="8"/>
     </row>
   </sheetData>
   <mergeCells count="38">
-    <mergeCell ref="C23:C25"/>
-    <mergeCell ref="C14:C22"/>
-    <mergeCell ref="D10:D12"/>
-    <mergeCell ref="D14:D16"/>
-    <mergeCell ref="E14:E16"/>
-    <mergeCell ref="D17:D19"/>
-    <mergeCell ref="C4:C13"/>
-    <mergeCell ref="D7:D9"/>
-    <mergeCell ref="E7:E9"/>
-    <mergeCell ref="F23:F25"/>
-    <mergeCell ref="E23:E25"/>
-    <mergeCell ref="D23:D25"/>
-    <mergeCell ref="F14:F16"/>
-    <mergeCell ref="E17:E19"/>
-    <mergeCell ref="F17:F19"/>
-    <mergeCell ref="D20:D22"/>
-    <mergeCell ref="E20:E22"/>
-    <mergeCell ref="F20:F22"/>
+    <mergeCell ref="F7:F9"/>
+    <mergeCell ref="D4:D6"/>
+    <mergeCell ref="E4:E6"/>
+    <mergeCell ref="F4:F6"/>
+    <mergeCell ref="I14:I16"/>
+    <mergeCell ref="F10:F12"/>
+    <mergeCell ref="E10:E12"/>
     <mergeCell ref="I17:I19"/>
     <mergeCell ref="I20:I22"/>
     <mergeCell ref="I23:I25"/>
@@ -986,13 +988,24 @@
     <mergeCell ref="H17:H19"/>
     <mergeCell ref="H20:H22"/>
     <mergeCell ref="H23:H25"/>
-    <mergeCell ref="F7:F9"/>
-    <mergeCell ref="D4:D6"/>
-    <mergeCell ref="E4:E6"/>
-    <mergeCell ref="F4:F6"/>
-    <mergeCell ref="I14:I16"/>
-    <mergeCell ref="F10:F12"/>
-    <mergeCell ref="E10:E12"/>
+    <mergeCell ref="F23:F25"/>
+    <mergeCell ref="E23:E25"/>
+    <mergeCell ref="D23:D25"/>
+    <mergeCell ref="F14:F16"/>
+    <mergeCell ref="E17:E19"/>
+    <mergeCell ref="F17:F19"/>
+    <mergeCell ref="D20:D22"/>
+    <mergeCell ref="E20:E22"/>
+    <mergeCell ref="F20:F22"/>
+    <mergeCell ref="C23:C25"/>
+    <mergeCell ref="C14:C22"/>
+    <mergeCell ref="D10:D12"/>
+    <mergeCell ref="D14:D16"/>
+    <mergeCell ref="E14:E16"/>
+    <mergeCell ref="D17:D19"/>
+    <mergeCell ref="C4:C13"/>
+    <mergeCell ref="D7:D9"/>
+    <mergeCell ref="E7:E9"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup scale="55" orientation="landscape" r:id="rId1"/>

</xml_diff>

<commit_message>
Add booking use case
</commit_message>
<xml_diff>
--- a/docs/Methods.xlsx
+++ b/docs/Methods.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\API\ConferenceRoomBooking\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F660ECCF-40BB-4EA8-A329-857B7DD370B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7025B8AD-5765-4A92-BFA6-5B6DD43EAFF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="4185" windowWidth="29040" windowHeight="15720" xr2:uid="{290D68D7-7384-40BB-827B-CD27B026537C}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="48">
   <si>
     <t>Method</t>
   </si>
@@ -94,9 +94,6 @@
   </si>
   <si>
     <t>ExistsOverlappingBookingAsync()</t>
-  </si>
-  <si>
-    <t>AddAsync() SaveChangesAsync()</t>
   </si>
   <si>
     <t xml:space="preserve">BookingService </t>
@@ -279,10 +276,10 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -605,7 +602,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="C3:I25"/>
+  <dimension ref="C3:I26"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="0" style="1" hidden="1" customWidth="1"/>
@@ -621,7 +618,7 @@
   <sheetData>
     <row r="3" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C3" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>0</v>
@@ -636,142 +633,142 @@
         <v>3</v>
       </c>
       <c r="H3" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="I3" s="3" t="s">
         <v>34</v>
-      </c>
-      <c r="I3" s="3" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="4" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C4" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="D4" s="9" t="s">
+      <c r="D4" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="9" t="s">
+      <c r="E4" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="F4" s="9" t="s">
+      <c r="F4" s="8" t="s">
         <v>7</v>
       </c>
       <c r="G4" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="H4" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="I4" s="9" t="s">
-        <v>43</v>
+      <c r="H4" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="I4" s="8" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="5" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C5" s="10"/>
-      <c r="D5" s="9"/>
-      <c r="E5" s="9"/>
-      <c r="F5" s="9"/>
+      <c r="D5" s="8"/>
+      <c r="E5" s="8"/>
+      <c r="F5" s="8"/>
       <c r="G5" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="H5" s="9"/>
-      <c r="I5" s="9"/>
+      <c r="H5" s="8"/>
+      <c r="I5" s="8"/>
     </row>
     <row r="6" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C6" s="10"/>
-      <c r="D6" s="9"/>
-      <c r="E6" s="9"/>
-      <c r="F6" s="9"/>
+      <c r="D6" s="8"/>
+      <c r="E6" s="8"/>
+      <c r="F6" s="8"/>
       <c r="G6" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="H6" s="9"/>
-      <c r="I6" s="9"/>
+      <c r="H6" s="8"/>
+      <c r="I6" s="8"/>
     </row>
     <row r="7" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C7" s="10"/>
-      <c r="D7" s="9" t="s">
+      <c r="D7" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="E7" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="F7" s="9" t="s">
-        <v>22</v>
+      <c r="E7" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="F7" s="8" t="s">
+        <v>21</v>
       </c>
       <c r="G7" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="H7" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="I7" s="9" t="s">
-        <v>44</v>
+        <v>45</v>
+      </c>
+      <c r="H7" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="I7" s="8" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="8" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C8" s="10"/>
-      <c r="D8" s="9"/>
-      <c r="E8" s="9"/>
-      <c r="F8" s="9"/>
+      <c r="D8" s="8"/>
+      <c r="E8" s="8"/>
+      <c r="F8" s="8"/>
       <c r="G8" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="H8" s="9"/>
-      <c r="I8" s="9"/>
+      <c r="H8" s="8"/>
+      <c r="I8" s="8"/>
     </row>
     <row r="9" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C9" s="10"/>
-      <c r="D9" s="9"/>
-      <c r="E9" s="9"/>
-      <c r="F9" s="9"/>
+      <c r="D9" s="8"/>
+      <c r="E9" s="8"/>
+      <c r="F9" s="8"/>
       <c r="G9" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="H9" s="9"/>
-      <c r="I9" s="9"/>
+      <c r="H9" s="8"/>
+      <c r="I9" s="8"/>
     </row>
     <row r="10" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C10" s="10"/>
-      <c r="D10" s="9" t="s">
+      <c r="D10" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="E10" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="F10" s="9" t="s">
-        <v>22</v>
+      <c r="E10" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="F10" s="8" t="s">
+        <v>21</v>
       </c>
       <c r="G10" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="H10" s="9" t="s">
-        <v>38</v>
-      </c>
-      <c r="I10" s="9" t="s">
-        <v>45</v>
+      <c r="H10" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="I10" s="8" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="11" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C11" s="10"/>
-      <c r="D11" s="9"/>
-      <c r="E11" s="9"/>
-      <c r="F11" s="9"/>
+      <c r="D11" s="8"/>
+      <c r="E11" s="8"/>
+      <c r="F11" s="8"/>
       <c r="G11" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="H11" s="9"/>
-      <c r="I11" s="9"/>
+      <c r="H11" s="8"/>
+      <c r="I11" s="8"/>
     </row>
     <row r="12" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C12" s="10"/>
-      <c r="D12" s="9"/>
-      <c r="E12" s="9"/>
-      <c r="F12" s="9"/>
+      <c r="D12" s="8"/>
+      <c r="E12" s="8"/>
+      <c r="F12" s="8"/>
       <c r="G12" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="H12" s="9"/>
-      <c r="I12" s="9"/>
+        <v>32</v>
+      </c>
+      <c r="H12" s="8"/>
+      <c r="I12" s="8"/>
     </row>
     <row r="13" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C13" s="10"/>
@@ -779,205 +776,227 @@
         <v>15</v>
       </c>
       <c r="E13" s="7" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G13" s="7" t="s">
         <v>13</v>
       </c>
       <c r="H13" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="I13" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="I13" s="7" t="s">
-        <v>48</v>
-      </c>
     </row>
     <row r="14" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C14" s="9" t="s">
+      <c r="C14" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="D14" s="9" t="s">
+      <c r="D14" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="E14" s="9" t="s">
-        <v>30</v>
-      </c>
-      <c r="F14" s="9" t="s">
-        <v>24</v>
+      <c r="E14" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="F14" s="8" t="s">
+        <v>23</v>
       </c>
       <c r="G14" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="H14" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="I14" s="9" t="s">
-        <v>39</v>
+      <c r="H14" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="I14" s="8" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="15" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C15" s="9"/>
-      <c r="D15" s="9"/>
-      <c r="E15" s="9"/>
-      <c r="F15" s="9"/>
+      <c r="C15" s="8"/>
+      <c r="D15" s="8"/>
+      <c r="E15" s="8"/>
+      <c r="F15" s="8"/>
       <c r="G15" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="H15" s="9"/>
-      <c r="I15" s="9"/>
+      <c r="H15" s="8"/>
+      <c r="I15" s="8"/>
     </row>
     <row r="16" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C16" s="9"/>
-      <c r="D16" s="9"/>
-      <c r="E16" s="9"/>
-      <c r="F16" s="9"/>
+      <c r="C16" s="8"/>
+      <c r="D16" s="8"/>
+      <c r="E16" s="8"/>
+      <c r="F16" s="8"/>
       <c r="G16" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="H16" s="9"/>
-      <c r="I16" s="9"/>
+      <c r="H16" s="8"/>
+      <c r="I16" s="8"/>
     </row>
     <row r="17" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C17" s="9"/>
-      <c r="D17" s="9" t="s">
+      <c r="C17" s="8"/>
+      <c r="D17" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="E17" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="F17" s="9" t="s">
-        <v>25</v>
+      <c r="E17" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="F17" s="8" t="s">
+        <v>24</v>
       </c>
       <c r="G17" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="H17" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="I17" s="9" t="s">
-        <v>40</v>
+      <c r="H17" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="I17" s="8" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="18" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C18" s="9"/>
-      <c r="D18" s="9"/>
-      <c r="E18" s="9"/>
-      <c r="F18" s="9"/>
+      <c r="C18" s="8"/>
+      <c r="D18" s="8"/>
+      <c r="E18" s="8"/>
+      <c r="F18" s="8"/>
       <c r="G18" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="H18" s="9"/>
-      <c r="I18" s="9"/>
+      <c r="H18" s="8"/>
+      <c r="I18" s="8"/>
     </row>
     <row r="19" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C19" s="9"/>
-      <c r="D19" s="9"/>
-      <c r="E19" s="9"/>
-      <c r="F19" s="9"/>
+      <c r="C19" s="8"/>
+      <c r="D19" s="8"/>
+      <c r="E19" s="8"/>
+      <c r="F19" s="8"/>
       <c r="G19" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="H19" s="9"/>
-      <c r="I19" s="9"/>
+      <c r="H19" s="8"/>
+      <c r="I19" s="8"/>
     </row>
     <row r="20" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C20" s="9"/>
-      <c r="D20" s="9" t="s">
+      <c r="C20" s="8"/>
+      <c r="D20" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="E20" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="F20" s="9" t="s">
-        <v>25</v>
+      <c r="E20" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="F20" s="8" t="s">
+        <v>24</v>
       </c>
       <c r="G20" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="H20" s="9" t="s">
-        <v>38</v>
-      </c>
-      <c r="I20" s="9" t="s">
-        <v>41</v>
+      <c r="H20" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="I20" s="8" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="21" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C21" s="9"/>
-      <c r="D21" s="9"/>
-      <c r="E21" s="9"/>
-      <c r="F21" s="9"/>
+      <c r="C21" s="8"/>
+      <c r="D21" s="8"/>
+      <c r="E21" s="8"/>
+      <c r="F21" s="8"/>
       <c r="G21" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="H21" s="9"/>
-      <c r="I21" s="9"/>
+      <c r="H21" s="8"/>
+      <c r="I21" s="8"/>
     </row>
     <row r="22" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C22" s="9"/>
-      <c r="D22" s="9"/>
-      <c r="E22" s="9"/>
-      <c r="F22" s="9"/>
+      <c r="C22" s="8"/>
+      <c r="D22" s="8"/>
+      <c r="E22" s="8"/>
+      <c r="F22" s="8"/>
       <c r="G22" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="H22" s="9"/>
-      <c r="I22" s="9"/>
+      <c r="H22" s="8"/>
+      <c r="I22" s="8"/>
     </row>
     <row r="23" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C23" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="D23" s="8" t="s">
+      <c r="C23" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="D23" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="E23" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="F23" s="8" t="s">
-        <v>26</v>
+      <c r="E23" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="F23" s="9" t="s">
+        <v>25</v>
       </c>
       <c r="G23" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="H23" s="8"/>
-      <c r="I23" s="8"/>
+      <c r="H23" s="9"/>
+      <c r="I23" s="9"/>
     </row>
     <row r="24" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C24" s="8"/>
-      <c r="D24" s="8"/>
-      <c r="E24" s="8"/>
-      <c r="F24" s="8"/>
+      <c r="C24" s="9"/>
+      <c r="D24" s="9"/>
+      <c r="E24" s="9"/>
+      <c r="F24" s="9"/>
       <c r="G24" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="H24" s="8"/>
-      <c r="I24" s="8"/>
+      <c r="H24" s="9"/>
+      <c r="I24" s="9"/>
     </row>
     <row r="25" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C25" s="8"/>
-      <c r="D25" s="8"/>
-      <c r="E25" s="8"/>
-      <c r="F25" s="8"/>
+      <c r="C25" s="9"/>
+      <c r="D25" s="9"/>
+      <c r="E25" s="9"/>
+      <c r="F25" s="9"/>
       <c r="G25" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="H25" s="8"/>
-      <c r="I25" s="8"/>
+        <v>9</v>
+      </c>
+      <c r="H25" s="9"/>
+      <c r="I25" s="9"/>
+    </row>
+    <row r="26" spans="3:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C26" s="9"/>
+      <c r="D26" s="9"/>
+      <c r="E26" s="9"/>
+      <c r="F26" s="9"/>
+      <c r="G26" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="H26" s="9"/>
+      <c r="I26" s="9"/>
     </row>
   </sheetData>
   <mergeCells count="38">
-    <mergeCell ref="F7:F9"/>
-    <mergeCell ref="D4:D6"/>
-    <mergeCell ref="E4:E6"/>
-    <mergeCell ref="F4:F6"/>
-    <mergeCell ref="I14:I16"/>
-    <mergeCell ref="F10:F12"/>
-    <mergeCell ref="E10:E12"/>
+    <mergeCell ref="C23:C26"/>
+    <mergeCell ref="C14:C22"/>
+    <mergeCell ref="D10:D12"/>
+    <mergeCell ref="D14:D16"/>
+    <mergeCell ref="E14:E16"/>
+    <mergeCell ref="D17:D19"/>
+    <mergeCell ref="C4:C13"/>
+    <mergeCell ref="D7:D9"/>
+    <mergeCell ref="E7:E9"/>
+    <mergeCell ref="F23:F26"/>
+    <mergeCell ref="E23:E26"/>
+    <mergeCell ref="D23:D26"/>
+    <mergeCell ref="F14:F16"/>
+    <mergeCell ref="E17:E19"/>
+    <mergeCell ref="F17:F19"/>
+    <mergeCell ref="D20:D22"/>
+    <mergeCell ref="E20:E22"/>
+    <mergeCell ref="F20:F22"/>
     <mergeCell ref="I17:I19"/>
     <mergeCell ref="I20:I22"/>
-    <mergeCell ref="I23:I25"/>
+    <mergeCell ref="I23:I26"/>
     <mergeCell ref="H4:H6"/>
     <mergeCell ref="I4:I6"/>
     <mergeCell ref="H7:H9"/>
@@ -987,25 +1006,14 @@
     <mergeCell ref="H14:H16"/>
     <mergeCell ref="H17:H19"/>
     <mergeCell ref="H20:H22"/>
-    <mergeCell ref="H23:H25"/>
-    <mergeCell ref="F23:F25"/>
-    <mergeCell ref="E23:E25"/>
-    <mergeCell ref="D23:D25"/>
-    <mergeCell ref="F14:F16"/>
-    <mergeCell ref="E17:E19"/>
-    <mergeCell ref="F17:F19"/>
-    <mergeCell ref="D20:D22"/>
-    <mergeCell ref="E20:E22"/>
-    <mergeCell ref="F20:F22"/>
-    <mergeCell ref="C23:C25"/>
-    <mergeCell ref="C14:C22"/>
-    <mergeCell ref="D10:D12"/>
-    <mergeCell ref="D14:D16"/>
-    <mergeCell ref="E14:E16"/>
-    <mergeCell ref="D17:D19"/>
-    <mergeCell ref="C4:C13"/>
-    <mergeCell ref="D7:D9"/>
-    <mergeCell ref="E7:E9"/>
+    <mergeCell ref="H23:H26"/>
+    <mergeCell ref="F7:F9"/>
+    <mergeCell ref="D4:D6"/>
+    <mergeCell ref="E4:E6"/>
+    <mergeCell ref="F4:F6"/>
+    <mergeCell ref="I14:I16"/>
+    <mergeCell ref="F10:F12"/>
+    <mergeCell ref="E10:E12"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup scale="55" orientation="landscape" r:id="rId1"/>

</xml_diff>